<commit_message>
Self-host logos; fix FX bug at pipeline source; remove delisted tickers; inline citations
</commit_message>
<xml_diff>
--- a/Mizan_Outreach_Tracker.xlsx
+++ b/Mizan_Outreach_Tracker.xlsx
@@ -21,9 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -219,7 +220,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -360,6 +361,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1885,19 +1889,25 @@
         </is>
       </c>
       <c r="F24" s="42" t="n"/>
-      <c r="G24" s="42" t="n"/>
-      <c r="H24" s="42" t="n"/>
+      <c r="G24" s="42" t="inlineStr">
+        <is>
+          <t>REPLIED</t>
+        </is>
+      </c>
+      <c r="H24" s="48" t="n">
+        <v>46182</v>
+      </c>
       <c r="I24" s="42" t="n"/>
       <c r="J24" s="42" t="inlineStr">
         <is>
-          <t>Pending — sent today</t>
+          <t>ENGAGED — replied 'please dm at 51162640' (WhatsApp)</t>
         </is>
       </c>
       <c r="K24" s="42" t="n"/>
       <c r="L24" s="42" t="n"/>
       <c r="M24" s="42" t="inlineStr">
         <is>
-          <t>Wait 3-7 days; reply within 24h if they respond</t>
+          <t>WhatsApp 51162640 with one-paragraph blurb</t>
         </is>
       </c>
       <c r="N24" s="42" t="inlineStr">
@@ -2235,132 +2245,516 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="22">
-      <c r="A30" s="28" t="n"/>
-      <c r="B30" s="28" t="n"/>
-      <c r="C30" s="28" t="n"/>
-      <c r="D30" s="28" t="n"/>
-      <c r="E30" s="28" t="n"/>
-      <c r="F30" s="28" t="n"/>
-      <c r="G30" s="28" t="n"/>
-      <c r="H30" s="28" t="n"/>
-      <c r="I30" s="28" t="n"/>
-      <c r="J30" s="28" t="n"/>
-      <c r="K30" s="28" t="n"/>
-      <c r="L30" s="28" t="n"/>
-      <c r="M30" s="28" t="n"/>
-      <c r="N30" s="28" t="n"/>
+      <c r="A30" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>Terence Chong, Prof. (CUHK IGEF / Economics)</t>
+        </is>
+      </c>
+      <c r="C30" s="42" t="inlineStr">
+        <is>
+          <t>Email (Gordon direct)</t>
+        </is>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+      <c r="E30" s="42" t="inlineStr">
+        <is>
+          <t>CUHK economist; Islamic economics/finance angle</t>
+        </is>
+      </c>
+      <c r="F30" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="42" t="inlineStr">
+        <is>
+          <t>REPLIED</t>
+        </is>
+      </c>
+      <c r="H30" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="I30" s="42" t="inlineStr">
+        <is>
+          <t>Thanks for the email and happy to see your work</t>
+        </is>
+      </c>
+      <c r="J30" s="42" t="inlineStr">
+        <is>
+          <t>MEETING — Zoom Mon 15 Jun, 3pm proposed</t>
+        </is>
+      </c>
+      <c r="K30" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M30" s="42" t="inlineStr">
+        <is>
+          <t>Send Zoom link + confirm 3pm</t>
+        </is>
+      </c>
+      <c r="N30" s="42" t="inlineStr">
+        <is>
+          <t>Replied within ~1.5h of email. Senior CUHK faculty.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="22">
-      <c r="A31" s="28" t="n"/>
-      <c r="B31" s="28" t="n"/>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="28" t="n"/>
-      <c r="E31" s="28" t="n"/>
-      <c r="F31" s="28" t="n"/>
-      <c r="G31" s="28" t="n"/>
-      <c r="H31" s="28" t="n"/>
-      <c r="I31" s="28" t="n"/>
-      <c r="J31" s="28" t="n"/>
-      <c r="K31" s="28" t="n"/>
-      <c r="L31" s="28" t="n"/>
-      <c r="M31" s="28" t="n"/>
-      <c r="N31" s="28" t="n"/>
+      <c r="A31" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>Pawee Jenweeranon (CUHK Law)</t>
+        </is>
+      </c>
+      <c r="C31" s="42" t="inlineStr">
+        <is>
+          <t>Email (Gordon direct)</t>
+        </is>
+      </c>
+      <c r="D31" s="42" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+      <c r="E31" s="42" t="inlineStr">
+        <is>
+          <t>CUHK Law; Islamic finance law / transparency</t>
+        </is>
+      </c>
+      <c r="F31" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="42" t="inlineStr">
+        <is>
+          <t>REPLIED</t>
+        </is>
+      </c>
+      <c r="H31" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="I31" s="42" t="inlineStr">
+        <is>
+          <t>It sounds like a very interesting project... happy to have a chat</t>
+        </is>
+      </c>
+      <c r="J31" s="42" t="inlineStr">
+        <is>
+          <t>ENGAGED — will send Zoom slots</t>
+        </is>
+      </c>
+      <c r="K31" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M31" s="42" t="inlineStr">
+        <is>
+          <t>Add WhatsApp +66639094725; await slots</t>
+        </is>
+      </c>
+      <c r="N31" s="42" t="inlineStr">
+        <is>
+          <t>Shared WeChat paweejen + WhatsApp. Warm.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="22">
-      <c r="A32" s="28" t="n"/>
-      <c r="B32" s="28" t="n"/>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="28" t="n"/>
-      <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
-      <c r="H32" s="28" t="n"/>
-      <c r="I32" s="28" t="n"/>
-      <c r="J32" s="28" t="n"/>
-      <c r="K32" s="28" t="n"/>
-      <c r="L32" s="28" t="n"/>
-      <c r="M32" s="28" t="n"/>
-      <c r="N32" s="28" t="n"/>
+      <c r="A32" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
+          <t>Prof. Frankel (CUHK CSIC)</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="inlineStr">
+        <is>
+          <t>Email (Gordon direct)</t>
+        </is>
+      </c>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+      <c r="E32" s="42" t="inlineStr">
+        <is>
+          <t>CUHK CSIC</t>
+        </is>
+      </c>
+      <c r="F32" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H32" s="42" t="inlineStr"/>
+      <c r="I32" s="42" t="inlineStr"/>
+      <c r="J32" s="42" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K32" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M32" s="42" t="inlineStr">
+        <is>
+          <t>Await reply</t>
+        </is>
+      </c>
+      <c r="N32" s="42" t="inlineStr">
+        <is>
+          <t>One of the Day-11 CUHK academic emails.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="22">
-      <c r="A33" s="28" t="n"/>
-      <c r="B33" s="28" t="n"/>
-      <c r="C33" s="28" t="n"/>
-      <c r="D33" s="28" t="n"/>
-      <c r="E33" s="28" t="n"/>
-      <c r="F33" s="28" t="n"/>
-      <c r="G33" s="28" t="n"/>
-      <c r="H33" s="28" t="n"/>
-      <c r="I33" s="28" t="n"/>
-      <c r="J33" s="28" t="n"/>
-      <c r="K33" s="28" t="n"/>
-      <c r="L33" s="28" t="n"/>
-      <c r="M33" s="28" t="n"/>
-      <c r="N33" s="28" t="n"/>
+      <c r="A33" s="42" t="n"/>
+      <c r="B33" s="42" t="inlineStr">
+        <is>
+          <t>Dr. HoiYan Kwok (CUHK Finance for Society)</t>
+        </is>
+      </c>
+      <c r="C33" s="42" t="inlineStr">
+        <is>
+          <t>Email (Gordon direct)</t>
+        </is>
+      </c>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+      <c r="E33" s="42" t="inlineStr">
+        <is>
+          <t>Finance for Society Research Centre</t>
+        </is>
+      </c>
+      <c r="F33" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="42" t="inlineStr">
+        <is>
+          <t>NOT SENT</t>
+        </is>
+      </c>
+      <c r="H33" s="42" t="inlineStr"/>
+      <c r="I33" s="42" t="inlineStr"/>
+      <c r="J33" s="42" t="inlineStr">
+        <is>
+          <t>DRAFT READY — not yet sent</t>
+        </is>
+      </c>
+      <c r="K33" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M33" s="42" t="inlineStr">
+        <is>
+          <t>Send drafted email (OUTREACH_SEND_QUEUE)</t>
+        </is>
+      </c>
+      <c r="N33" s="42" t="inlineStr">
+        <is>
+          <t>4th CUHK academic; draft prepared, pending send.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="22">
-      <c r="A34" s="28" t="n"/>
-      <c r="B34" s="28" t="n"/>
-      <c r="C34" s="28" t="n"/>
-      <c r="D34" s="28" t="n"/>
-      <c r="E34" s="28" t="n"/>
-      <c r="F34" s="28" t="n"/>
-      <c r="G34" s="28" t="n"/>
-      <c r="H34" s="28" t="n"/>
-      <c r="I34" s="28" t="n"/>
-      <c r="J34" s="28" t="n"/>
-      <c r="K34" s="28" t="n"/>
-      <c r="L34" s="28" t="n"/>
-      <c r="M34" s="28" t="n"/>
-      <c r="N34" s="28" t="n"/>
+      <c r="A34" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>The Islamic Union of Hong Kong</t>
+        </is>
+      </c>
+      <c r="C34" s="42" t="inlineStr">
+        <is>
+          <t>Instagram DM (@iuhkorg)</t>
+        </is>
+      </c>
+      <c r="D34" s="42" t="inlineStr">
+        <is>
+          <t>Community org</t>
+        </is>
+      </c>
+      <c r="E34" s="42" t="inlineStr">
+        <is>
+          <t>HK masjid/union; sent 3-asks + banner image</t>
+        </is>
+      </c>
+      <c r="F34" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="42" t="inlineStr">
+        <is>
+          <t>REPLIED</t>
+        </is>
+      </c>
+      <c r="H34" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="I34" s="42" t="inlineStr">
+        <is>
+          <t>Wsalam, please leave your contact or WhatsApp number</t>
+        </is>
+      </c>
+      <c r="J34" s="42" t="inlineStr">
+        <is>
+          <t>ENGAGED — wants contact/WhatsApp</t>
+        </is>
+      </c>
+      <c r="K34" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M34" s="42" t="inlineStr">
+        <is>
+          <t>Send WhatsApp / contact</t>
+        </is>
+      </c>
+      <c r="N34" s="42" t="inlineStr">
+        <is>
+          <t>Replied requesting contact.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="22">
-      <c r="A35" s="28" t="n"/>
-      <c r="B35" s="28" t="n"/>
-      <c r="C35" s="28" t="n"/>
-      <c r="D35" s="28" t="n"/>
-      <c r="E35" s="28" t="n"/>
-      <c r="F35" s="28" t="n"/>
-      <c r="G35" s="28" t="n"/>
-      <c r="H35" s="28" t="n"/>
-      <c r="I35" s="28" t="n"/>
-      <c r="J35" s="28" t="n"/>
-      <c r="K35" s="28" t="n"/>
-      <c r="L35" s="28" t="n"/>
-      <c r="M35" s="28" t="n"/>
-      <c r="N35" s="28" t="n"/>
+      <c r="A35" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B35" s="42" t="inlineStr">
+        <is>
+          <t>Muslim Council of Hong Kong</t>
+        </is>
+      </c>
+      <c r="C35" s="42" t="inlineStr">
+        <is>
+          <t>Instagram DM (@mchk)</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>Community org</t>
+        </is>
+      </c>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>HK Muslim council</t>
+        </is>
+      </c>
+      <c r="F35" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H35" s="42" t="inlineStr"/>
+      <c r="I35" s="42" t="inlineStr"/>
+      <c r="J35" s="42" t="inlineStr">
+        <is>
+          <t>Pending — DM sent</t>
+        </is>
+      </c>
+      <c r="K35" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M35" s="42" t="inlineStr">
+        <is>
+          <t>Await reply</t>
+        </is>
+      </c>
+      <c r="N35" s="42" t="inlineStr">
+        <is>
+          <t>Day-11 community blitz.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="22">
-      <c r="A36" s="28" t="n"/>
-      <c r="B36" s="28" t="n"/>
-      <c r="C36" s="28" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="28" t="n"/>
-      <c r="F36" s="28" t="n"/>
-      <c r="G36" s="28" t="n"/>
-      <c r="H36" s="28" t="n"/>
-      <c r="I36" s="28" t="n"/>
-      <c r="J36" s="28" t="n"/>
-      <c r="K36" s="28" t="n"/>
-      <c r="L36" s="28" t="n"/>
-      <c r="M36" s="28" t="n"/>
-      <c r="N36" s="28" t="n"/>
+      <c r="A36" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>Council of Hong Kong Muslims</t>
+        </is>
+      </c>
+      <c r="C36" s="42" t="inlineStr">
+        <is>
+          <t>Instagram DM</t>
+        </is>
+      </c>
+      <c r="D36" s="42" t="inlineStr">
+        <is>
+          <t>Community org</t>
+        </is>
+      </c>
+      <c r="E36" s="42" t="inlineStr">
+        <is>
+          <t>HK Muslim community org</t>
+        </is>
+      </c>
+      <c r="F36" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H36" s="42" t="inlineStr"/>
+      <c r="I36" s="42" t="inlineStr"/>
+      <c r="J36" s="42" t="inlineStr">
+        <is>
+          <t>Pending — DM sent</t>
+        </is>
+      </c>
+      <c r="K36" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M36" s="42" t="inlineStr">
+        <is>
+          <t>Await reply</t>
+        </is>
+      </c>
+      <c r="N36" s="42" t="inlineStr">
+        <is>
+          <t>Day-11 community blitz.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="22">
-      <c r="A37" s="28" t="n"/>
-      <c r="B37" s="28" t="n"/>
-      <c r="C37" s="28" t="n"/>
-      <c r="D37" s="28" t="n"/>
-      <c r="E37" s="28" t="n"/>
-      <c r="F37" s="28" t="n"/>
-      <c r="G37" s="28" t="n"/>
-      <c r="H37" s="28" t="n"/>
-      <c r="I37" s="28" t="n"/>
-      <c r="J37" s="28" t="n"/>
-      <c r="K37" s="28" t="n"/>
-      <c r="L37" s="28" t="n"/>
-      <c r="M37" s="28" t="n"/>
-      <c r="N37" s="28" t="n"/>
+      <c r="A37" s="48" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B37" s="42" t="inlineStr">
+        <is>
+          <t>Hong Kong India Club</t>
+        </is>
+      </c>
+      <c r="C37" s="42" t="inlineStr">
+        <is>
+          <t>Instagram DM</t>
+        </is>
+      </c>
+      <c r="D37" s="42" t="inlineStr">
+        <is>
+          <t>Community org</t>
+        </is>
+      </c>
+      <c r="E37" s="42" t="inlineStr">
+        <is>
+          <t>HK South-Asian community</t>
+        </is>
+      </c>
+      <c r="F37" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H37" s="42" t="inlineStr"/>
+      <c r="I37" s="42" t="inlineStr"/>
+      <c r="J37" s="42" t="inlineStr">
+        <is>
+          <t>Pending — DM sent</t>
+        </is>
+      </c>
+      <c r="K37" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" s="42" t="inlineStr">
+        <is>
+          <t>Await reply</t>
+        </is>
+      </c>
+      <c r="N37" s="42" t="inlineStr">
+        <is>
+          <t>Day-11 community blitz.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="22">
       <c r="A38" s="28" t="n"/>
@@ -3506,6 +3900,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="22">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -3527,6 +3922,7 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="22">
       <c r="A7" s="33" t="inlineStr">
         <is>
@@ -3843,12 +4239,26 @@
           <t>Day 12</t>
         </is>
       </c>
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="28" t="n"/>
-      <c r="E21" s="28" t="n"/>
-      <c r="F21" s="28" t="n"/>
-      <c r="G21" s="28" t="n"/>
+      <c r="B21" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>Date 2026-06-09. THREE academics replied: Prof. Terence Chong (CUHK) -&gt; Zoom 15 Jun 3pm; Pawee Jenweeranon (CUHK Law) -&gt; sending slots, shared WhatsApp; Frankel emailed (pending). 4 HK community orgs DM'd (Muslim Council, Council of HK Muslims, Islamic Union, HK India Club). Islamic Union + HKIYA replied asking for WhatsApp. Dr. Kwok email drafted, not yet sent. 0 unprompted shares.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="22">
       <c r="A22" s="38" t="inlineStr">

</xml_diff>